<commit_message>
Add design doc; document supporting tasks per lead (Tareas sheet)
Add docs/DESIGN.md (architecture, principles, workflow + tech-stack
Mermaid sketches) as the bridge between the PRD and CLAUDE.md.

Add a Tareas sheet so owners document supporting tasks per lead
measure: WIG | Lead | Tarea | Responsable | Estado (Pendiente/En
curso/Hecho, with dropdown validation). build_wig.py generates it with
seed examples; marcador.html parseTareas() reads it and the TV shows
"Tareas de soporte" in each lead's detail drill-down; migrate_data.py
carries real rows forward; tests + CLAUDE.md contract updated. make
test green (8/8).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Tablero_WIG_4DX_GBM.xlsx
+++ b/dist/Tablero_WIG_4DX_GBM.xlsx
@@ -24,7 +24,8 @@
     <sheet name="2027" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="2028" sheetId="15" state="visible" r:id="rId17"/>
     <sheet name="2029" sheetId="16" state="visible" r:id="rId18"/>
-    <sheet name="Instrucciones" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Tareas" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Instrucciones" sheetId="18" state="visible" r:id="rId20"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="258">
   <si>
     <t xml:space="preserve">Tablero 4DX — GBM Nicaragua</t>
   </si>
@@ -713,6 +714,42 @@
     <t xml:space="preserve">Backlog comprometido por semana (2029)</t>
   </si>
   <si>
+    <t xml:space="preserve">WIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tareas de soporte por lead: cada fila es una acción concreta que sostiene un lead measure. WIG = número de pestaña (1–12), Lead = 1–8. Aparecen en el detalle del lead en el televisor. Estado: Pendiente · En curso · Hecho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentar la oferta Smart User a 100 clientes en 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-Sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certificarse como Apple Authorized Service Provider para reparar equipos con mayor eficiencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Del - DEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantener siempre 50 equipos en bodega listos para colocar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cómo usar este tablero 4DX</t>
   </si>
   <si>
@@ -744,6 +781,18 @@
   </si>
   <si>
     <t xml:space="preserve">• Definan todos los leads en positivo (más = mejor) para que el % se lea igual en todos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAREAS DE SOPORTE (pestaña «Tareas»):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Cada fila es una acción concreta que sostiene un lead measure: WIG (1–12), Lead (1–8), la tarea, el responsable y el estado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Usen los desplegables de las columnas WIG, Lead y Estado (Pendiente · En curso · Hecho) para no salirse de rango.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Aparecen en el televisor al tocar el lead correspondiente (sección «Tareas de soporte» del detalle).</t>
   </si>
   <si>
     <t xml:space="preserve">CÓDIGO DE COLORES:</t>
@@ -1006,7 +1055,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="91">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1339,6 +1388,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1826,11 +1895,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="96901920"/>
-        <c:axId val="42734147"/>
+        <c:axId val="25181191"/>
+        <c:axId val="55061646"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="96901920"/>
+        <c:axId val="25181191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1863,7 +1932,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42734147"/>
+        <c:crossAx val="55061646"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1871,7 +1940,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42734147"/>
+        <c:axId val="55061646"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1914,7 +1983,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96901920"/>
+        <c:crossAx val="25181191"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2349,11 +2418,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78823596"/>
-        <c:axId val="60964993"/>
+        <c:axId val="83085169"/>
+        <c:axId val="42962334"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78823596"/>
+        <c:axId val="83085169"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2386,7 +2455,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60964993"/>
+        <c:crossAx val="42962334"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2394,7 +2463,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60964993"/>
+        <c:axId val="42962334"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2437,7 +2506,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78823596"/>
+        <c:crossAx val="83085169"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2872,11 +2941,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="77850473"/>
-        <c:axId val="41608192"/>
+        <c:axId val="50237234"/>
+        <c:axId val="85542"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="77850473"/>
+        <c:axId val="50237234"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2909,7 +2978,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41608192"/>
+        <c:crossAx val="85542"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2917,7 +2986,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41608192"/>
+        <c:axId val="85542"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2960,7 +3029,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77850473"/>
+        <c:crossAx val="50237234"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3395,11 +3464,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="65842525"/>
-        <c:axId val="98210661"/>
+        <c:axId val="20371311"/>
+        <c:axId val="70146442"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="65842525"/>
+        <c:axId val="20371311"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3432,7 +3501,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98210661"/>
+        <c:crossAx val="70146442"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3440,7 +3509,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98210661"/>
+        <c:axId val="70146442"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3483,7 +3552,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65842525"/>
+        <c:crossAx val="20371311"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3918,11 +3987,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="83319684"/>
-        <c:axId val="30883696"/>
+        <c:axId val="77367358"/>
+        <c:axId val="75861377"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83319684"/>
+        <c:axId val="77367358"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3955,7 +4024,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30883696"/>
+        <c:crossAx val="75861377"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3963,7 +4032,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30883696"/>
+        <c:axId val="75861377"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4006,7 +4075,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83319684"/>
+        <c:crossAx val="77367358"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4540,11 +4609,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="22086008"/>
-        <c:axId val="78427543"/>
+        <c:axId val="93723319"/>
+        <c:axId val="8361812"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="22086008"/>
+        <c:axId val="93723319"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4577,7 +4646,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78427543"/>
+        <c:crossAx val="8361812"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4585,7 +4654,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78427543"/>
+        <c:axId val="8361812"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4628,7 +4697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22086008"/>
+        <c:crossAx val="93723319"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5162,11 +5231,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="29554109"/>
-        <c:axId val="60147358"/>
+        <c:axId val="61560205"/>
+        <c:axId val="76154393"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="29554109"/>
+        <c:axId val="61560205"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5199,7 +5268,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60147358"/>
+        <c:crossAx val="76154393"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5207,7 +5276,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60147358"/>
+        <c:axId val="76154393"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5250,7 +5319,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29554109"/>
+        <c:crossAx val="61560205"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5784,11 +5853,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="48827494"/>
-        <c:axId val="11020097"/>
+        <c:axId val="9482190"/>
+        <c:axId val="34185293"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48827494"/>
+        <c:axId val="9482190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5821,7 +5890,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11020097"/>
+        <c:crossAx val="34185293"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5829,7 +5898,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11020097"/>
+        <c:axId val="34185293"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5872,7 +5941,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48827494"/>
+        <c:crossAx val="9482190"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6493,11 +6562,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="10709604"/>
-        <c:axId val="65566530"/>
+        <c:axId val="97878061"/>
+        <c:axId val="70995789"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="10709604"/>
+        <c:axId val="97878061"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6530,7 +6599,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65566530"/>
+        <c:crossAx val="70995789"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6538,7 +6607,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65566530"/>
+        <c:axId val="70995789"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6581,7 +6650,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10709604"/>
+        <c:crossAx val="97878061"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7358,11 +7427,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="48883252"/>
-        <c:axId val="3004145"/>
+        <c:axId val="28403620"/>
+        <c:axId val="80151398"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48883252"/>
+        <c:axId val="28403620"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7395,7 +7464,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3004145"/>
+        <c:crossAx val="80151398"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7403,7 +7472,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3004145"/>
+        <c:axId val="80151398"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7446,7 +7515,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48883252"/>
+        <c:crossAx val="28403620"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8691,11 +8760,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="14571691"/>
-        <c:axId val="11913909"/>
+        <c:axId val="47511578"/>
+        <c:axId val="11054847"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="14571691"/>
+        <c:axId val="47511578"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8728,7 +8797,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11913909"/>
+        <c:crossAx val="11054847"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8736,7 +8805,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11913909"/>
+        <c:axId val="11054847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8779,7 +8848,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14571691"/>
+        <c:crossAx val="47511578"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9781,11 +9850,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="79581754"/>
-        <c:axId val="51134895"/>
+        <c:axId val="29593116"/>
+        <c:axId val="8345055"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="79581754"/>
+        <c:axId val="29593116"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9818,7 +9887,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51134895"/>
+        <c:crossAx val="8345055"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9826,7 +9895,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51134895"/>
+        <c:axId val="8345055"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9869,7 +9938,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79581754"/>
+        <c:crossAx val="29593116"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11114,11 +11183,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="69436279"/>
-        <c:axId val="85933130"/>
+        <c:axId val="37765702"/>
+        <c:axId val="10574670"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="69436279"/>
+        <c:axId val="37765702"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11151,7 +11220,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85933130"/>
+        <c:crossAx val="10574670"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11159,7 +11228,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85933130"/>
+        <c:axId val="10574670"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11202,7 +11271,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69436279"/>
+        <c:crossAx val="37765702"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12204,11 +12273,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40618697"/>
-        <c:axId val="65861906"/>
+        <c:axId val="27660775"/>
+        <c:axId val="70384001"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40618697"/>
+        <c:axId val="27660775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12241,7 +12310,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65861906"/>
+        <c:crossAx val="70384001"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12249,7 +12318,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65861906"/>
+        <c:axId val="70384001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12292,7 +12361,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40618697"/>
+        <c:crossAx val="27660775"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13117,11 +13186,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="92658915"/>
-        <c:axId val="75012643"/>
+        <c:axId val="94034608"/>
+        <c:axId val="58959669"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="92658915"/>
+        <c:axId val="94034608"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13154,7 +13223,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75012643"/>
+        <c:crossAx val="58959669"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13162,7 +13231,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75012643"/>
+        <c:axId val="58959669"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13205,7 +13274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92658915"/>
+        <c:crossAx val="94034608"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13640,11 +13709,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="27877360"/>
-        <c:axId val="46938438"/>
+        <c:axId val="88031251"/>
+        <c:axId val="18490518"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="27877360"/>
+        <c:axId val="88031251"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13677,7 +13746,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46938438"/>
+        <c:crossAx val="18490518"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13685,7 +13754,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46938438"/>
+        <c:axId val="18490518"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13728,7 +13797,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27877360"/>
+        <c:crossAx val="88031251"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -26785,95 +26854,1055 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:G121"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="262.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="83" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="84" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="D2" s="85" t="s">
+        <v>231</v>
+      </c>
+      <c r="E2" s="84" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="85" t="s">
+        <v>233</v>
+      </c>
+      <c r="D3" s="85" t="s">
+        <v>234</v>
+      </c>
+      <c r="E3" s="84" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="84" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="85" t="s">
+        <v>236</v>
+      </c>
+      <c r="D4" s="85" t="s">
+        <v>234</v>
+      </c>
+      <c r="E4" s="84" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="86"/>
+      <c r="B5" s="86"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="86"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="84"/>
+      <c r="B6" s="84"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="84"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="86"/>
+      <c r="B7" s="86"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="86"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="84"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="85"/>
+      <c r="D8" s="85"/>
+      <c r="E8" s="84"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="86"/>
+      <c r="B9" s="86"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="87"/>
+      <c r="E9" s="86"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="84"/>
+      <c r="B10" s="84"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="84"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="86"/>
+      <c r="B11" s="86"/>
+      <c r="C11" s="87"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="86"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="84"/>
+      <c r="B12" s="84"/>
+      <c r="C12" s="85"/>
+      <c r="D12" s="85"/>
+      <c r="E12" s="84"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="86"/>
+      <c r="B13" s="86"/>
+      <c r="C13" s="87"/>
+      <c r="D13" s="87"/>
+      <c r="E13" s="86"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="84"/>
+      <c r="B14" s="84"/>
+      <c r="C14" s="85"/>
+      <c r="D14" s="85"/>
+      <c r="E14" s="84"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="86"/>
+      <c r="B15" s="86"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="87"/>
+      <c r="E15" s="86"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="84"/>
+      <c r="B16" s="84"/>
+      <c r="C16" s="85"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="84"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="86"/>
+      <c r="B17" s="86"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="86"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="84"/>
+      <c r="B18" s="84"/>
+      <c r="C18" s="85"/>
+      <c r="D18" s="85"/>
+      <c r="E18" s="84"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="86"/>
+      <c r="B19" s="86"/>
+      <c r="C19" s="87"/>
+      <c r="D19" s="87"/>
+      <c r="E19" s="86"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="84"/>
+      <c r="B20" s="84"/>
+      <c r="C20" s="85"/>
+      <c r="D20" s="85"/>
+      <c r="E20" s="84"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="86"/>
+      <c r="B21" s="86"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="86"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="84"/>
+      <c r="B22" s="84"/>
+      <c r="C22" s="85"/>
+      <c r="D22" s="85"/>
+      <c r="E22" s="84"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="86"/>
+      <c r="B23" s="86"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="86"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="84"/>
+      <c r="B24" s="84"/>
+      <c r="C24" s="85"/>
+      <c r="D24" s="85"/>
+      <c r="E24" s="84"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="86"/>
+      <c r="B25" s="86"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="86"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="84"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="85"/>
+      <c r="D26" s="85"/>
+      <c r="E26" s="84"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="86"/>
+      <c r="B27" s="86"/>
+      <c r="C27" s="87"/>
+      <c r="D27" s="87"/>
+      <c r="E27" s="86"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="84"/>
+      <c r="B28" s="84"/>
+      <c r="C28" s="85"/>
+      <c r="D28" s="85"/>
+      <c r="E28" s="84"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="86"/>
+      <c r="B29" s="86"/>
+      <c r="C29" s="87"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="86"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="84"/>
+      <c r="B30" s="84"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="84"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="86"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="86"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="84"/>
+      <c r="B32" s="84"/>
+      <c r="C32" s="85"/>
+      <c r="D32" s="85"/>
+      <c r="E32" s="84"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="86"/>
+      <c r="B33" s="86"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="86"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="84"/>
+      <c r="B34" s="84"/>
+      <c r="C34" s="85"/>
+      <c r="D34" s="85"/>
+      <c r="E34" s="84"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="86"/>
+      <c r="B35" s="86"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="87"/>
+      <c r="E35" s="86"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="84"/>
+      <c r="B36" s="84"/>
+      <c r="C36" s="85"/>
+      <c r="D36" s="85"/>
+      <c r="E36" s="84"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="86"/>
+      <c r="B37" s="86"/>
+      <c r="C37" s="87"/>
+      <c r="D37" s="87"/>
+      <c r="E37" s="86"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="84"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="85"/>
+      <c r="D38" s="85"/>
+      <c r="E38" s="84"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="86"/>
+      <c r="B39" s="86"/>
+      <c r="C39" s="87"/>
+      <c r="D39" s="87"/>
+      <c r="E39" s="86"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="84"/>
+      <c r="B40" s="84"/>
+      <c r="C40" s="85"/>
+      <c r="D40" s="85"/>
+      <c r="E40" s="84"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="86"/>
+      <c r="B41" s="86"/>
+      <c r="C41" s="87"/>
+      <c r="D41" s="87"/>
+      <c r="E41" s="86"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="84"/>
+      <c r="B42" s="84"/>
+      <c r="C42" s="85"/>
+      <c r="D42" s="85"/>
+      <c r="E42" s="84"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="86"/>
+      <c r="B43" s="86"/>
+      <c r="C43" s="87"/>
+      <c r="D43" s="87"/>
+      <c r="E43" s="86"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="84"/>
+      <c r="B44" s="84"/>
+      <c r="C44" s="85"/>
+      <c r="D44" s="85"/>
+      <c r="E44" s="84"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="86"/>
+      <c r="B45" s="86"/>
+      <c r="C45" s="87"/>
+      <c r="D45" s="87"/>
+      <c r="E45" s="86"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="84"/>
+      <c r="B46" s="84"/>
+      <c r="C46" s="85"/>
+      <c r="D46" s="85"/>
+      <c r="E46" s="84"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="86"/>
+      <c r="B47" s="86"/>
+      <c r="C47" s="87"/>
+      <c r="D47" s="87"/>
+      <c r="E47" s="86"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="84"/>
+      <c r="B48" s="84"/>
+      <c r="C48" s="85"/>
+      <c r="D48" s="85"/>
+      <c r="E48" s="84"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="86"/>
+      <c r="B49" s="86"/>
+      <c r="C49" s="87"/>
+      <c r="D49" s="87"/>
+      <c r="E49" s="86"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="84"/>
+      <c r="B50" s="84"/>
+      <c r="C50" s="85"/>
+      <c r="D50" s="85"/>
+      <c r="E50" s="84"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="86"/>
+      <c r="B51" s="86"/>
+      <c r="C51" s="87"/>
+      <c r="D51" s="87"/>
+      <c r="E51" s="86"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="84"/>
+      <c r="B52" s="84"/>
+      <c r="C52" s="85"/>
+      <c r="D52" s="85"/>
+      <c r="E52" s="84"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="86"/>
+      <c r="B53" s="86"/>
+      <c r="C53" s="87"/>
+      <c r="D53" s="87"/>
+      <c r="E53" s="86"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="84"/>
+      <c r="B54" s="84"/>
+      <c r="C54" s="85"/>
+      <c r="D54" s="85"/>
+      <c r="E54" s="84"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="86"/>
+      <c r="B55" s="86"/>
+      <c r="C55" s="87"/>
+      <c r="D55" s="87"/>
+      <c r="E55" s="86"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="84"/>
+      <c r="B56" s="84"/>
+      <c r="C56" s="85"/>
+      <c r="D56" s="85"/>
+      <c r="E56" s="84"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="86"/>
+      <c r="B57" s="86"/>
+      <c r="C57" s="87"/>
+      <c r="D57" s="87"/>
+      <c r="E57" s="86"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="84"/>
+      <c r="B58" s="84"/>
+      <c r="C58" s="85"/>
+      <c r="D58" s="85"/>
+      <c r="E58" s="84"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="86"/>
+      <c r="B59" s="86"/>
+      <c r="C59" s="87"/>
+      <c r="D59" s="87"/>
+      <c r="E59" s="86"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="84"/>
+      <c r="B60" s="84"/>
+      <c r="C60" s="85"/>
+      <c r="D60" s="85"/>
+      <c r="E60" s="84"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="86"/>
+      <c r="B61" s="86"/>
+      <c r="C61" s="87"/>
+      <c r="D61" s="87"/>
+      <c r="E61" s="86"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="84"/>
+      <c r="B62" s="84"/>
+      <c r="C62" s="85"/>
+      <c r="D62" s="85"/>
+      <c r="E62" s="84"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="86"/>
+      <c r="B63" s="86"/>
+      <c r="C63" s="87"/>
+      <c r="D63" s="87"/>
+      <c r="E63" s="86"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="84"/>
+      <c r="B64" s="84"/>
+      <c r="C64" s="85"/>
+      <c r="D64" s="85"/>
+      <c r="E64" s="84"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="86"/>
+      <c r="B65" s="86"/>
+      <c r="C65" s="87"/>
+      <c r="D65" s="87"/>
+      <c r="E65" s="86"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="84"/>
+      <c r="B66" s="84"/>
+      <c r="C66" s="85"/>
+      <c r="D66" s="85"/>
+      <c r="E66" s="84"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="86"/>
+      <c r="B67" s="86"/>
+      <c r="C67" s="87"/>
+      <c r="D67" s="87"/>
+      <c r="E67" s="86"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="84"/>
+      <c r="B68" s="84"/>
+      <c r="C68" s="85"/>
+      <c r="D68" s="85"/>
+      <c r="E68" s="84"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="86"/>
+      <c r="B69" s="86"/>
+      <c r="C69" s="87"/>
+      <c r="D69" s="87"/>
+      <c r="E69" s="86"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="84"/>
+      <c r="B70" s="84"/>
+      <c r="C70" s="85"/>
+      <c r="D70" s="85"/>
+      <c r="E70" s="84"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="86"/>
+      <c r="B71" s="86"/>
+      <c r="C71" s="87"/>
+      <c r="D71" s="87"/>
+      <c r="E71" s="86"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="84"/>
+      <c r="B72" s="84"/>
+      <c r="C72" s="85"/>
+      <c r="D72" s="85"/>
+      <c r="E72" s="84"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="86"/>
+      <c r="B73" s="86"/>
+      <c r="C73" s="87"/>
+      <c r="D73" s="87"/>
+      <c r="E73" s="86"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="84"/>
+      <c r="B74" s="84"/>
+      <c r="C74" s="85"/>
+      <c r="D74" s="85"/>
+      <c r="E74" s="84"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="86"/>
+      <c r="B75" s="86"/>
+      <c r="C75" s="87"/>
+      <c r="D75" s="87"/>
+      <c r="E75" s="86"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="84"/>
+      <c r="B76" s="84"/>
+      <c r="C76" s="85"/>
+      <c r="D76" s="85"/>
+      <c r="E76" s="84"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="86"/>
+      <c r="B77" s="86"/>
+      <c r="C77" s="87"/>
+      <c r="D77" s="87"/>
+      <c r="E77" s="86"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="84"/>
+      <c r="B78" s="84"/>
+      <c r="C78" s="85"/>
+      <c r="D78" s="85"/>
+      <c r="E78" s="84"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="86"/>
+      <c r="B79" s="86"/>
+      <c r="C79" s="87"/>
+      <c r="D79" s="87"/>
+      <c r="E79" s="86"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="84"/>
+      <c r="B80" s="84"/>
+      <c r="C80" s="85"/>
+      <c r="D80" s="85"/>
+      <c r="E80" s="84"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="86"/>
+      <c r="B81" s="86"/>
+      <c r="C81" s="87"/>
+      <c r="D81" s="87"/>
+      <c r="E81" s="86"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="84"/>
+      <c r="B82" s="84"/>
+      <c r="C82" s="85"/>
+      <c r="D82" s="85"/>
+      <c r="E82" s="84"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="86"/>
+      <c r="B83" s="86"/>
+      <c r="C83" s="87"/>
+      <c r="D83" s="87"/>
+      <c r="E83" s="86"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="84"/>
+      <c r="B84" s="84"/>
+      <c r="C84" s="85"/>
+      <c r="D84" s="85"/>
+      <c r="E84" s="84"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="86"/>
+      <c r="B85" s="86"/>
+      <c r="C85" s="87"/>
+      <c r="D85" s="87"/>
+      <c r="E85" s="86"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="84"/>
+      <c r="B86" s="84"/>
+      <c r="C86" s="85"/>
+      <c r="D86" s="85"/>
+      <c r="E86" s="84"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="86"/>
+      <c r="B87" s="86"/>
+      <c r="C87" s="87"/>
+      <c r="D87" s="87"/>
+      <c r="E87" s="86"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="84"/>
+      <c r="B88" s="84"/>
+      <c r="C88" s="85"/>
+      <c r="D88" s="85"/>
+      <c r="E88" s="84"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="86"/>
+      <c r="B89" s="86"/>
+      <c r="C89" s="87"/>
+      <c r="D89" s="87"/>
+      <c r="E89" s="86"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="84"/>
+      <c r="B90" s="84"/>
+      <c r="C90" s="85"/>
+      <c r="D90" s="85"/>
+      <c r="E90" s="84"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="86"/>
+      <c r="B91" s="86"/>
+      <c r="C91" s="87"/>
+      <c r="D91" s="87"/>
+      <c r="E91" s="86"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="84"/>
+      <c r="B92" s="84"/>
+      <c r="C92" s="85"/>
+      <c r="D92" s="85"/>
+      <c r="E92" s="84"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="86"/>
+      <c r="B93" s="86"/>
+      <c r="C93" s="87"/>
+      <c r="D93" s="87"/>
+      <c r="E93" s="86"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="84"/>
+      <c r="B94" s="84"/>
+      <c r="C94" s="85"/>
+      <c r="D94" s="85"/>
+      <c r="E94" s="84"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="86"/>
+      <c r="B95" s="86"/>
+      <c r="C95" s="87"/>
+      <c r="D95" s="87"/>
+      <c r="E95" s="86"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="84"/>
+      <c r="B96" s="84"/>
+      <c r="C96" s="85"/>
+      <c r="D96" s="85"/>
+      <c r="E96" s="84"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="86"/>
+      <c r="B97" s="86"/>
+      <c r="C97" s="87"/>
+      <c r="D97" s="87"/>
+      <c r="E97" s="86"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="84"/>
+      <c r="B98" s="84"/>
+      <c r="C98" s="85"/>
+      <c r="D98" s="85"/>
+      <c r="E98" s="84"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="86"/>
+      <c r="B99" s="86"/>
+      <c r="C99" s="87"/>
+      <c r="D99" s="87"/>
+      <c r="E99" s="86"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="84"/>
+      <c r="B100" s="84"/>
+      <c r="C100" s="85"/>
+      <c r="D100" s="85"/>
+      <c r="E100" s="84"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="86"/>
+      <c r="B101" s="86"/>
+      <c r="C101" s="87"/>
+      <c r="D101" s="87"/>
+      <c r="E101" s="86"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="84"/>
+      <c r="B102" s="84"/>
+      <c r="C102" s="85"/>
+      <c r="D102" s="85"/>
+      <c r="E102" s="84"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="86"/>
+      <c r="B103" s="86"/>
+      <c r="C103" s="87"/>
+      <c r="D103" s="87"/>
+      <c r="E103" s="86"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="84"/>
+      <c r="B104" s="84"/>
+      <c r="C104" s="85"/>
+      <c r="D104" s="85"/>
+      <c r="E104" s="84"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="86"/>
+      <c r="B105" s="86"/>
+      <c r="C105" s="87"/>
+      <c r="D105" s="87"/>
+      <c r="E105" s="86"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="84"/>
+      <c r="B106" s="84"/>
+      <c r="C106" s="85"/>
+      <c r="D106" s="85"/>
+      <c r="E106" s="84"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="86"/>
+      <c r="B107" s="86"/>
+      <c r="C107" s="87"/>
+      <c r="D107" s="87"/>
+      <c r="E107" s="86"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="84"/>
+      <c r="B108" s="84"/>
+      <c r="C108" s="85"/>
+      <c r="D108" s="85"/>
+      <c r="E108" s="84"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="86"/>
+      <c r="B109" s="86"/>
+      <c r="C109" s="87"/>
+      <c r="D109" s="87"/>
+      <c r="E109" s="86"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="84"/>
+      <c r="B110" s="84"/>
+      <c r="C110" s="85"/>
+      <c r="D110" s="85"/>
+      <c r="E110" s="84"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="86"/>
+      <c r="B111" s="86"/>
+      <c r="C111" s="87"/>
+      <c r="D111" s="87"/>
+      <c r="E111" s="86"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="84"/>
+      <c r="B112" s="84"/>
+      <c r="C112" s="85"/>
+      <c r="D112" s="85"/>
+      <c r="E112" s="84"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="86"/>
+      <c r="B113" s="86"/>
+      <c r="C113" s="87"/>
+      <c r="D113" s="87"/>
+      <c r="E113" s="86"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="84"/>
+      <c r="B114" s="84"/>
+      <c r="C114" s="85"/>
+      <c r="D114" s="85"/>
+      <c r="E114" s="84"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="86"/>
+      <c r="B115" s="86"/>
+      <c r="C115" s="87"/>
+      <c r="D115" s="87"/>
+      <c r="E115" s="86"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="84"/>
+      <c r="B116" s="84"/>
+      <c r="C116" s="85"/>
+      <c r="D116" s="85"/>
+      <c r="E116" s="84"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="86"/>
+      <c r="B117" s="86"/>
+      <c r="C117" s="87"/>
+      <c r="D117" s="87"/>
+      <c r="E117" s="86"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="84"/>
+      <c r="B118" s="84"/>
+      <c r="C118" s="85"/>
+      <c r="D118" s="85"/>
+      <c r="E118" s="84"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="86"/>
+      <c r="B119" s="86"/>
+      <c r="C119" s="87"/>
+      <c r="D119" s="87"/>
+      <c r="E119" s="86"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="84"/>
+      <c r="B120" s="84"/>
+      <c r="C120" s="85"/>
+      <c r="D120" s="85"/>
+      <c r="E120" s="84"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="86"/>
+      <c r="B121" s="86"/>
+      <c r="C121" s="87"/>
+      <c r="D121" s="87"/>
+      <c r="E121" s="86"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E121">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Hecho" dxfId="0">
+      <formula>NOT(ISERROR(SEARCH("Hecho",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="En curso" dxfId="1">
+      <formula>NOT(ISERROR(SEARCH("En curso",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Pendiente" dxfId="2">
+      <formula>NOT(ISERROR(SEARCH("Pendiente",E2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A2:A121" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B121" type="list">
+      <formula1>"1,2,3,4,5,6,7,8"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E121" type="list">
+      <formula1>"Pendiente,En curso,Hecho"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="83" t="s">
-        <v>225</v>
+      <c r="A1" s="88" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="84" t="s">
-        <v>226</v>
+      <c r="A3" s="89" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="85" t="s">
-        <v>227</v>
+      <c r="A4" s="90" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="85" t="s">
-        <v>228</v>
+      <c r="A5" s="90" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="85" t="s">
-        <v>229</v>
+      <c r="A6" s="90" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="85" t="s">
-        <v>230</v>
+      <c r="A7" s="90" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="84" t="s">
-        <v>231</v>
+      <c r="A9" s="89" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="85" t="s">
-        <v>232</v>
+      <c r="A10" s="90" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="85" t="s">
-        <v>233</v>
+      <c r="A11" s="90" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="85" t="s">
-        <v>234</v>
+      <c r="A12" s="90" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="85" t="s">
-        <v>235</v>
+      <c r="A13" s="90" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="84" t="s">
-        <v>236</v>
+      <c r="A15" s="89" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="85" t="s">
-        <v>237</v>
+      <c r="A16" s="90" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="85" t="s">
-        <v>238</v>
+      <c r="A17" s="90" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="85" t="s">
-        <v>239</v>
+      <c r="A18" s="90" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="84" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="85" t="s">
-        <v>241</v>
+      <c r="A20" s="89" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="90" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="90" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="90" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="89" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="90" t="s">
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add design doc; document supporting tasks per lead (Tareas sheet) (#10)
Add docs/DESIGN.md (architecture, principles, workflow + tech-stack
Mermaid sketches) as the bridge between the PRD and CLAUDE.md.

Add a Tareas sheet so owners document supporting tasks per lead
measure: WIG | Lead | Tarea | Responsable | Estado (Pendiente/En
curso/Hecho, with dropdown validation). build_wig.py generates it with
seed examples; marcador.html parseTareas() reads it and the TV shows
"Tareas de soporte" in each lead's detail drill-down; migrate_data.py
carries real rows forward; tests + CLAUDE.md contract updated. make
test green (8/8).

Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dist/Tablero_WIG_4DX_GBM.xlsx
+++ b/dist/Tablero_WIG_4DX_GBM.xlsx
@@ -24,7 +24,8 @@
     <sheet name="2027" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="2028" sheetId="15" state="visible" r:id="rId17"/>
     <sheet name="2029" sheetId="16" state="visible" r:id="rId18"/>
-    <sheet name="Instrucciones" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Tareas" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Instrucciones" sheetId="18" state="visible" r:id="rId20"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="258">
   <si>
     <t xml:space="preserve">Tablero 4DX — GBM Nicaragua</t>
   </si>
@@ -713,6 +714,42 @@
     <t xml:space="preserve">Backlog comprometido por semana (2029)</t>
   </si>
   <si>
+    <t xml:space="preserve">WIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tareas de soporte por lead: cada fila es una acción concreta que sostiene un lead measure. WIG = número de pestaña (1–12), Lead = 1–8. Aparecen en el detalle del lead en el televisor. Estado: Pendiente · En curso · Hecho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentar la oferta Smart User a 100 clientes en 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-Sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certificarse como Apple Authorized Service Provider para reparar equipos con mayor eficiencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Del - DEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantener siempre 50 equipos en bodega listos para colocar</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cómo usar este tablero 4DX</t>
   </si>
   <si>
@@ -744,6 +781,18 @@
   </si>
   <si>
     <t xml:space="preserve">• Definan todos los leads en positivo (más = mejor) para que el % se lea igual en todos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAREAS DE SOPORTE (pestaña «Tareas»):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Cada fila es una acción concreta que sostiene un lead measure: WIG (1–12), Lead (1–8), la tarea, el responsable y el estado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Usen los desplegables de las columnas WIG, Lead y Estado (Pendiente · En curso · Hecho) para no salirse de rango.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Aparecen en el televisor al tocar el lead correspondiente (sección «Tareas de soporte» del detalle).</t>
   </si>
   <si>
     <t xml:space="preserve">CÓDIGO DE COLORES:</t>
@@ -1006,7 +1055,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="91">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1339,6 +1388,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1826,11 +1895,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="96901920"/>
-        <c:axId val="42734147"/>
+        <c:axId val="25181191"/>
+        <c:axId val="55061646"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="96901920"/>
+        <c:axId val="25181191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1863,7 +1932,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42734147"/>
+        <c:crossAx val="55061646"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1871,7 +1940,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42734147"/>
+        <c:axId val="55061646"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1914,7 +1983,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96901920"/>
+        <c:crossAx val="25181191"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2349,11 +2418,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78823596"/>
-        <c:axId val="60964993"/>
+        <c:axId val="83085169"/>
+        <c:axId val="42962334"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78823596"/>
+        <c:axId val="83085169"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2386,7 +2455,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60964993"/>
+        <c:crossAx val="42962334"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2394,7 +2463,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60964993"/>
+        <c:axId val="42962334"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2437,7 +2506,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78823596"/>
+        <c:crossAx val="83085169"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2872,11 +2941,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="77850473"/>
-        <c:axId val="41608192"/>
+        <c:axId val="50237234"/>
+        <c:axId val="85542"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="77850473"/>
+        <c:axId val="50237234"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2909,7 +2978,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41608192"/>
+        <c:crossAx val="85542"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2917,7 +2986,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41608192"/>
+        <c:axId val="85542"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2960,7 +3029,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77850473"/>
+        <c:crossAx val="50237234"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3395,11 +3464,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="65842525"/>
-        <c:axId val="98210661"/>
+        <c:axId val="20371311"/>
+        <c:axId val="70146442"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="65842525"/>
+        <c:axId val="20371311"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3432,7 +3501,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98210661"/>
+        <c:crossAx val="70146442"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3440,7 +3509,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98210661"/>
+        <c:axId val="70146442"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3483,7 +3552,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65842525"/>
+        <c:crossAx val="20371311"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3918,11 +3987,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="83319684"/>
-        <c:axId val="30883696"/>
+        <c:axId val="77367358"/>
+        <c:axId val="75861377"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83319684"/>
+        <c:axId val="77367358"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3955,7 +4024,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30883696"/>
+        <c:crossAx val="75861377"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3963,7 +4032,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30883696"/>
+        <c:axId val="75861377"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4006,7 +4075,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83319684"/>
+        <c:crossAx val="77367358"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4540,11 +4609,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="22086008"/>
-        <c:axId val="78427543"/>
+        <c:axId val="93723319"/>
+        <c:axId val="8361812"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="22086008"/>
+        <c:axId val="93723319"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4577,7 +4646,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78427543"/>
+        <c:crossAx val="8361812"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4585,7 +4654,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78427543"/>
+        <c:axId val="8361812"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4628,7 +4697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22086008"/>
+        <c:crossAx val="93723319"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5162,11 +5231,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="29554109"/>
-        <c:axId val="60147358"/>
+        <c:axId val="61560205"/>
+        <c:axId val="76154393"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="29554109"/>
+        <c:axId val="61560205"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5199,7 +5268,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60147358"/>
+        <c:crossAx val="76154393"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5207,7 +5276,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60147358"/>
+        <c:axId val="76154393"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5250,7 +5319,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29554109"/>
+        <c:crossAx val="61560205"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5784,11 +5853,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="48827494"/>
-        <c:axId val="11020097"/>
+        <c:axId val="9482190"/>
+        <c:axId val="34185293"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48827494"/>
+        <c:axId val="9482190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5821,7 +5890,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11020097"/>
+        <c:crossAx val="34185293"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5829,7 +5898,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11020097"/>
+        <c:axId val="34185293"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5872,7 +5941,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48827494"/>
+        <c:crossAx val="9482190"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6493,11 +6562,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="10709604"/>
-        <c:axId val="65566530"/>
+        <c:axId val="97878061"/>
+        <c:axId val="70995789"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="10709604"/>
+        <c:axId val="97878061"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6530,7 +6599,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65566530"/>
+        <c:crossAx val="70995789"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6538,7 +6607,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65566530"/>
+        <c:axId val="70995789"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6581,7 +6650,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10709604"/>
+        <c:crossAx val="97878061"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7358,11 +7427,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="48883252"/>
-        <c:axId val="3004145"/>
+        <c:axId val="28403620"/>
+        <c:axId val="80151398"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48883252"/>
+        <c:axId val="28403620"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7395,7 +7464,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3004145"/>
+        <c:crossAx val="80151398"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7403,7 +7472,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3004145"/>
+        <c:axId val="80151398"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7446,7 +7515,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48883252"/>
+        <c:crossAx val="28403620"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8691,11 +8760,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="14571691"/>
-        <c:axId val="11913909"/>
+        <c:axId val="47511578"/>
+        <c:axId val="11054847"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="14571691"/>
+        <c:axId val="47511578"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8728,7 +8797,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11913909"/>
+        <c:crossAx val="11054847"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8736,7 +8805,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11913909"/>
+        <c:axId val="11054847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8779,7 +8848,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14571691"/>
+        <c:crossAx val="47511578"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9781,11 +9850,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="79581754"/>
-        <c:axId val="51134895"/>
+        <c:axId val="29593116"/>
+        <c:axId val="8345055"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="79581754"/>
+        <c:axId val="29593116"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9818,7 +9887,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51134895"/>
+        <c:crossAx val="8345055"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9826,7 +9895,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51134895"/>
+        <c:axId val="8345055"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9869,7 +9938,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79581754"/>
+        <c:crossAx val="29593116"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -11114,11 +11183,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="69436279"/>
-        <c:axId val="85933130"/>
+        <c:axId val="37765702"/>
+        <c:axId val="10574670"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="69436279"/>
+        <c:axId val="37765702"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11151,7 +11220,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85933130"/>
+        <c:crossAx val="10574670"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11159,7 +11228,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85933130"/>
+        <c:axId val="10574670"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11202,7 +11271,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69436279"/>
+        <c:crossAx val="37765702"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -12204,11 +12273,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40618697"/>
-        <c:axId val="65861906"/>
+        <c:axId val="27660775"/>
+        <c:axId val="70384001"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40618697"/>
+        <c:axId val="27660775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12241,7 +12310,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65861906"/>
+        <c:crossAx val="70384001"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -12249,7 +12318,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65861906"/>
+        <c:axId val="70384001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12292,7 +12361,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40618697"/>
+        <c:crossAx val="27660775"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13117,11 +13186,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="92658915"/>
-        <c:axId val="75012643"/>
+        <c:axId val="94034608"/>
+        <c:axId val="58959669"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="92658915"/>
+        <c:axId val="94034608"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13154,7 +13223,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75012643"/>
+        <c:crossAx val="58959669"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13162,7 +13231,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75012643"/>
+        <c:axId val="58959669"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13205,7 +13274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92658915"/>
+        <c:crossAx val="94034608"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -13640,11 +13709,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="27877360"/>
-        <c:axId val="46938438"/>
+        <c:axId val="88031251"/>
+        <c:axId val="18490518"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="27877360"/>
+        <c:axId val="88031251"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13677,7 +13746,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46938438"/>
+        <c:crossAx val="18490518"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13685,7 +13754,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46938438"/>
+        <c:axId val="18490518"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13728,7 +13797,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27877360"/>
+        <c:crossAx val="88031251"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -26785,95 +26854,1055 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:G121"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="262.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="83" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="84" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="D2" s="85" t="s">
+        <v>231</v>
+      </c>
+      <c r="E2" s="84" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="85" t="s">
+        <v>233</v>
+      </c>
+      <c r="D3" s="85" t="s">
+        <v>234</v>
+      </c>
+      <c r="E3" s="84" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="84" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="84" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" s="85" t="s">
+        <v>236</v>
+      </c>
+      <c r="D4" s="85" t="s">
+        <v>234</v>
+      </c>
+      <c r="E4" s="84" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="86"/>
+      <c r="B5" s="86"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="86"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="84"/>
+      <c r="B6" s="84"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="84"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="86"/>
+      <c r="B7" s="86"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="86"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="84"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="85"/>
+      <c r="D8" s="85"/>
+      <c r="E8" s="84"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="86"/>
+      <c r="B9" s="86"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="87"/>
+      <c r="E9" s="86"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="84"/>
+      <c r="B10" s="84"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="84"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="86"/>
+      <c r="B11" s="86"/>
+      <c r="C11" s="87"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="86"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="84"/>
+      <c r="B12" s="84"/>
+      <c r="C12" s="85"/>
+      <c r="D12" s="85"/>
+      <c r="E12" s="84"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="86"/>
+      <c r="B13" s="86"/>
+      <c r="C13" s="87"/>
+      <c r="D13" s="87"/>
+      <c r="E13" s="86"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="84"/>
+      <c r="B14" s="84"/>
+      <c r="C14" s="85"/>
+      <c r="D14" s="85"/>
+      <c r="E14" s="84"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="86"/>
+      <c r="B15" s="86"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="87"/>
+      <c r="E15" s="86"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="84"/>
+      <c r="B16" s="84"/>
+      <c r="C16" s="85"/>
+      <c r="D16" s="85"/>
+      <c r="E16" s="84"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="86"/>
+      <c r="B17" s="86"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="86"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="84"/>
+      <c r="B18" s="84"/>
+      <c r="C18" s="85"/>
+      <c r="D18" s="85"/>
+      <c r="E18" s="84"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="86"/>
+      <c r="B19" s="86"/>
+      <c r="C19" s="87"/>
+      <c r="D19" s="87"/>
+      <c r="E19" s="86"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="84"/>
+      <c r="B20" s="84"/>
+      <c r="C20" s="85"/>
+      <c r="D20" s="85"/>
+      <c r="E20" s="84"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="86"/>
+      <c r="B21" s="86"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="86"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="84"/>
+      <c r="B22" s="84"/>
+      <c r="C22" s="85"/>
+      <c r="D22" s="85"/>
+      <c r="E22" s="84"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="86"/>
+      <c r="B23" s="86"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="86"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="84"/>
+      <c r="B24" s="84"/>
+      <c r="C24" s="85"/>
+      <c r="D24" s="85"/>
+      <c r="E24" s="84"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="86"/>
+      <c r="B25" s="86"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="86"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="84"/>
+      <c r="B26" s="84"/>
+      <c r="C26" s="85"/>
+      <c r="D26" s="85"/>
+      <c r="E26" s="84"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="86"/>
+      <c r="B27" s="86"/>
+      <c r="C27" s="87"/>
+      <c r="D27" s="87"/>
+      <c r="E27" s="86"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="84"/>
+      <c r="B28" s="84"/>
+      <c r="C28" s="85"/>
+      <c r="D28" s="85"/>
+      <c r="E28" s="84"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="86"/>
+      <c r="B29" s="86"/>
+      <c r="C29" s="87"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="86"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="84"/>
+      <c r="B30" s="84"/>
+      <c r="C30" s="85"/>
+      <c r="D30" s="85"/>
+      <c r="E30" s="84"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="86"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="86"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="84"/>
+      <c r="B32" s="84"/>
+      <c r="C32" s="85"/>
+      <c r="D32" s="85"/>
+      <c r="E32" s="84"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="86"/>
+      <c r="B33" s="86"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="86"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="84"/>
+      <c r="B34" s="84"/>
+      <c r="C34" s="85"/>
+      <c r="D34" s="85"/>
+      <c r="E34" s="84"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="86"/>
+      <c r="B35" s="86"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="87"/>
+      <c r="E35" s="86"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="84"/>
+      <c r="B36" s="84"/>
+      <c r="C36" s="85"/>
+      <c r="D36" s="85"/>
+      <c r="E36" s="84"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="86"/>
+      <c r="B37" s="86"/>
+      <c r="C37" s="87"/>
+      <c r="D37" s="87"/>
+      <c r="E37" s="86"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="84"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="85"/>
+      <c r="D38" s="85"/>
+      <c r="E38" s="84"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="86"/>
+      <c r="B39" s="86"/>
+      <c r="C39" s="87"/>
+      <c r="D39" s="87"/>
+      <c r="E39" s="86"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="84"/>
+      <c r="B40" s="84"/>
+      <c r="C40" s="85"/>
+      <c r="D40" s="85"/>
+      <c r="E40" s="84"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="86"/>
+      <c r="B41" s="86"/>
+      <c r="C41" s="87"/>
+      <c r="D41" s="87"/>
+      <c r="E41" s="86"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="84"/>
+      <c r="B42" s="84"/>
+      <c r="C42" s="85"/>
+      <c r="D42" s="85"/>
+      <c r="E42" s="84"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="86"/>
+      <c r="B43" s="86"/>
+      <c r="C43" s="87"/>
+      <c r="D43" s="87"/>
+      <c r="E43" s="86"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="84"/>
+      <c r="B44" s="84"/>
+      <c r="C44" s="85"/>
+      <c r="D44" s="85"/>
+      <c r="E44" s="84"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="86"/>
+      <c r="B45" s="86"/>
+      <c r="C45" s="87"/>
+      <c r="D45" s="87"/>
+      <c r="E45" s="86"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="84"/>
+      <c r="B46" s="84"/>
+      <c r="C46" s="85"/>
+      <c r="D46" s="85"/>
+      <c r="E46" s="84"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="86"/>
+      <c r="B47" s="86"/>
+      <c r="C47" s="87"/>
+      <c r="D47" s="87"/>
+      <c r="E47" s="86"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="84"/>
+      <c r="B48" s="84"/>
+      <c r="C48" s="85"/>
+      <c r="D48" s="85"/>
+      <c r="E48" s="84"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="86"/>
+      <c r="B49" s="86"/>
+      <c r="C49" s="87"/>
+      <c r="D49" s="87"/>
+      <c r="E49" s="86"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="84"/>
+      <c r="B50" s="84"/>
+      <c r="C50" s="85"/>
+      <c r="D50" s="85"/>
+      <c r="E50" s="84"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="86"/>
+      <c r="B51" s="86"/>
+      <c r="C51" s="87"/>
+      <c r="D51" s="87"/>
+      <c r="E51" s="86"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="84"/>
+      <c r="B52" s="84"/>
+      <c r="C52" s="85"/>
+      <c r="D52" s="85"/>
+      <c r="E52" s="84"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="86"/>
+      <c r="B53" s="86"/>
+      <c r="C53" s="87"/>
+      <c r="D53" s="87"/>
+      <c r="E53" s="86"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="84"/>
+      <c r="B54" s="84"/>
+      <c r="C54" s="85"/>
+      <c r="D54" s="85"/>
+      <c r="E54" s="84"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="86"/>
+      <c r="B55" s="86"/>
+      <c r="C55" s="87"/>
+      <c r="D55" s="87"/>
+      <c r="E55" s="86"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="84"/>
+      <c r="B56" s="84"/>
+      <c r="C56" s="85"/>
+      <c r="D56" s="85"/>
+      <c r="E56" s="84"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="86"/>
+      <c r="B57" s="86"/>
+      <c r="C57" s="87"/>
+      <c r="D57" s="87"/>
+      <c r="E57" s="86"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="84"/>
+      <c r="B58" s="84"/>
+      <c r="C58" s="85"/>
+      <c r="D58" s="85"/>
+      <c r="E58" s="84"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="86"/>
+      <c r="B59" s="86"/>
+      <c r="C59" s="87"/>
+      <c r="D59" s="87"/>
+      <c r="E59" s="86"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="84"/>
+      <c r="B60" s="84"/>
+      <c r="C60" s="85"/>
+      <c r="D60" s="85"/>
+      <c r="E60" s="84"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="86"/>
+      <c r="B61" s="86"/>
+      <c r="C61" s="87"/>
+      <c r="D61" s="87"/>
+      <c r="E61" s="86"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="84"/>
+      <c r="B62" s="84"/>
+      <c r="C62" s="85"/>
+      <c r="D62" s="85"/>
+      <c r="E62" s="84"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="86"/>
+      <c r="B63" s="86"/>
+      <c r="C63" s="87"/>
+      <c r="D63" s="87"/>
+      <c r="E63" s="86"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="84"/>
+      <c r="B64" s="84"/>
+      <c r="C64" s="85"/>
+      <c r="D64" s="85"/>
+      <c r="E64" s="84"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="86"/>
+      <c r="B65" s="86"/>
+      <c r="C65" s="87"/>
+      <c r="D65" s="87"/>
+      <c r="E65" s="86"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="84"/>
+      <c r="B66" s="84"/>
+      <c r="C66" s="85"/>
+      <c r="D66" s="85"/>
+      <c r="E66" s="84"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="86"/>
+      <c r="B67" s="86"/>
+      <c r="C67" s="87"/>
+      <c r="D67" s="87"/>
+      <c r="E67" s="86"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="84"/>
+      <c r="B68" s="84"/>
+      <c r="C68" s="85"/>
+      <c r="D68" s="85"/>
+      <c r="E68" s="84"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="86"/>
+      <c r="B69" s="86"/>
+      <c r="C69" s="87"/>
+      <c r="D69" s="87"/>
+      <c r="E69" s="86"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="84"/>
+      <c r="B70" s="84"/>
+      <c r="C70" s="85"/>
+      <c r="D70" s="85"/>
+      <c r="E70" s="84"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="86"/>
+      <c r="B71" s="86"/>
+      <c r="C71" s="87"/>
+      <c r="D71" s="87"/>
+      <c r="E71" s="86"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="84"/>
+      <c r="B72" s="84"/>
+      <c r="C72" s="85"/>
+      <c r="D72" s="85"/>
+      <c r="E72" s="84"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="86"/>
+      <c r="B73" s="86"/>
+      <c r="C73" s="87"/>
+      <c r="D73" s="87"/>
+      <c r="E73" s="86"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="84"/>
+      <c r="B74" s="84"/>
+      <c r="C74" s="85"/>
+      <c r="D74" s="85"/>
+      <c r="E74" s="84"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="86"/>
+      <c r="B75" s="86"/>
+      <c r="C75" s="87"/>
+      <c r="D75" s="87"/>
+      <c r="E75" s="86"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="84"/>
+      <c r="B76" s="84"/>
+      <c r="C76" s="85"/>
+      <c r="D76" s="85"/>
+      <c r="E76" s="84"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="86"/>
+      <c r="B77" s="86"/>
+      <c r="C77" s="87"/>
+      <c r="D77" s="87"/>
+      <c r="E77" s="86"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="84"/>
+      <c r="B78" s="84"/>
+      <c r="C78" s="85"/>
+      <c r="D78" s="85"/>
+      <c r="E78" s="84"/>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="86"/>
+      <c r="B79" s="86"/>
+      <c r="C79" s="87"/>
+      <c r="D79" s="87"/>
+      <c r="E79" s="86"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="84"/>
+      <c r="B80" s="84"/>
+      <c r="C80" s="85"/>
+      <c r="D80" s="85"/>
+      <c r="E80" s="84"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="86"/>
+      <c r="B81" s="86"/>
+      <c r="C81" s="87"/>
+      <c r="D81" s="87"/>
+      <c r="E81" s="86"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="84"/>
+      <c r="B82" s="84"/>
+      <c r="C82" s="85"/>
+      <c r="D82" s="85"/>
+      <c r="E82" s="84"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="86"/>
+      <c r="B83" s="86"/>
+      <c r="C83" s="87"/>
+      <c r="D83" s="87"/>
+      <c r="E83" s="86"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="84"/>
+      <c r="B84" s="84"/>
+      <c r="C84" s="85"/>
+      <c r="D84" s="85"/>
+      <c r="E84" s="84"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="86"/>
+      <c r="B85" s="86"/>
+      <c r="C85" s="87"/>
+      <c r="D85" s="87"/>
+      <c r="E85" s="86"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="84"/>
+      <c r="B86" s="84"/>
+      <c r="C86" s="85"/>
+      <c r="D86" s="85"/>
+      <c r="E86" s="84"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="86"/>
+      <c r="B87" s="86"/>
+      <c r="C87" s="87"/>
+      <c r="D87" s="87"/>
+      <c r="E87" s="86"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="84"/>
+      <c r="B88" s="84"/>
+      <c r="C88" s="85"/>
+      <c r="D88" s="85"/>
+      <c r="E88" s="84"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="86"/>
+      <c r="B89" s="86"/>
+      <c r="C89" s="87"/>
+      <c r="D89" s="87"/>
+      <c r="E89" s="86"/>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="84"/>
+      <c r="B90" s="84"/>
+      <c r="C90" s="85"/>
+      <c r="D90" s="85"/>
+      <c r="E90" s="84"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="86"/>
+      <c r="B91" s="86"/>
+      <c r="C91" s="87"/>
+      <c r="D91" s="87"/>
+      <c r="E91" s="86"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="84"/>
+      <c r="B92" s="84"/>
+      <c r="C92" s="85"/>
+      <c r="D92" s="85"/>
+      <c r="E92" s="84"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="86"/>
+      <c r="B93" s="86"/>
+      <c r="C93" s="87"/>
+      <c r="D93" s="87"/>
+      <c r="E93" s="86"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="84"/>
+      <c r="B94" s="84"/>
+      <c r="C94" s="85"/>
+      <c r="D94" s="85"/>
+      <c r="E94" s="84"/>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="86"/>
+      <c r="B95" s="86"/>
+      <c r="C95" s="87"/>
+      <c r="D95" s="87"/>
+      <c r="E95" s="86"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="84"/>
+      <c r="B96" s="84"/>
+      <c r="C96" s="85"/>
+      <c r="D96" s="85"/>
+      <c r="E96" s="84"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="86"/>
+      <c r="B97" s="86"/>
+      <c r="C97" s="87"/>
+      <c r="D97" s="87"/>
+      <c r="E97" s="86"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="84"/>
+      <c r="B98" s="84"/>
+      <c r="C98" s="85"/>
+      <c r="D98" s="85"/>
+      <c r="E98" s="84"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="86"/>
+      <c r="B99" s="86"/>
+      <c r="C99" s="87"/>
+      <c r="D99" s="87"/>
+      <c r="E99" s="86"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="84"/>
+      <c r="B100" s="84"/>
+      <c r="C100" s="85"/>
+      <c r="D100" s="85"/>
+      <c r="E100" s="84"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="86"/>
+      <c r="B101" s="86"/>
+      <c r="C101" s="87"/>
+      <c r="D101" s="87"/>
+      <c r="E101" s="86"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="84"/>
+      <c r="B102" s="84"/>
+      <c r="C102" s="85"/>
+      <c r="D102" s="85"/>
+      <c r="E102" s="84"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="86"/>
+      <c r="B103" s="86"/>
+      <c r="C103" s="87"/>
+      <c r="D103" s="87"/>
+      <c r="E103" s="86"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="84"/>
+      <c r="B104" s="84"/>
+      <c r="C104" s="85"/>
+      <c r="D104" s="85"/>
+      <c r="E104" s="84"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="86"/>
+      <c r="B105" s="86"/>
+      <c r="C105" s="87"/>
+      <c r="D105" s="87"/>
+      <c r="E105" s="86"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="84"/>
+      <c r="B106" s="84"/>
+      <c r="C106" s="85"/>
+      <c r="D106" s="85"/>
+      <c r="E106" s="84"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="86"/>
+      <c r="B107" s="86"/>
+      <c r="C107" s="87"/>
+      <c r="D107" s="87"/>
+      <c r="E107" s="86"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="84"/>
+      <c r="B108" s="84"/>
+      <c r="C108" s="85"/>
+      <c r="D108" s="85"/>
+      <c r="E108" s="84"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="86"/>
+      <c r="B109" s="86"/>
+      <c r="C109" s="87"/>
+      <c r="D109" s="87"/>
+      <c r="E109" s="86"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="84"/>
+      <c r="B110" s="84"/>
+      <c r="C110" s="85"/>
+      <c r="D110" s="85"/>
+      <c r="E110" s="84"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="86"/>
+      <c r="B111" s="86"/>
+      <c r="C111" s="87"/>
+      <c r="D111" s="87"/>
+      <c r="E111" s="86"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="84"/>
+      <c r="B112" s="84"/>
+      <c r="C112" s="85"/>
+      <c r="D112" s="85"/>
+      <c r="E112" s="84"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="86"/>
+      <c r="B113" s="86"/>
+      <c r="C113" s="87"/>
+      <c r="D113" s="87"/>
+      <c r="E113" s="86"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="84"/>
+      <c r="B114" s="84"/>
+      <c r="C114" s="85"/>
+      <c r="D114" s="85"/>
+      <c r="E114" s="84"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="86"/>
+      <c r="B115" s="86"/>
+      <c r="C115" s="87"/>
+      <c r="D115" s="87"/>
+      <c r="E115" s="86"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="84"/>
+      <c r="B116" s="84"/>
+      <c r="C116" s="85"/>
+      <c r="D116" s="85"/>
+      <c r="E116" s="84"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="86"/>
+      <c r="B117" s="86"/>
+      <c r="C117" s="87"/>
+      <c r="D117" s="87"/>
+      <c r="E117" s="86"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="84"/>
+      <c r="B118" s="84"/>
+      <c r="C118" s="85"/>
+      <c r="D118" s="85"/>
+      <c r="E118" s="84"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="86"/>
+      <c r="B119" s="86"/>
+      <c r="C119" s="87"/>
+      <c r="D119" s="87"/>
+      <c r="E119" s="86"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="84"/>
+      <c r="B120" s="84"/>
+      <c r="C120" s="85"/>
+      <c r="D120" s="85"/>
+      <c r="E120" s="84"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="86"/>
+      <c r="B121" s="86"/>
+      <c r="C121" s="87"/>
+      <c r="D121" s="87"/>
+      <c r="E121" s="86"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:E121">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Hecho" dxfId="0">
+      <formula>NOT(ISERROR(SEARCH("Hecho",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="En curso" dxfId="1">
+      <formula>NOT(ISERROR(SEARCH("En curso",E2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Pendiente" dxfId="2">
+      <formula>NOT(ISERROR(SEARCH("Pendiente",E2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A2:A121" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,10,11,12"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B2:B121" type="list">
+      <formula1>"1,2,3,4,5,6,7,8"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E121" type="list">
+      <formula1>"Pendiente,En curso,Hecho"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="83" t="s">
-        <v>225</v>
+      <c r="A1" s="88" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="84" t="s">
-        <v>226</v>
+      <c r="A3" s="89" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="85" t="s">
-        <v>227</v>
+      <c r="A4" s="90" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="85" t="s">
-        <v>228</v>
+      <c r="A5" s="90" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="85" t="s">
-        <v>229</v>
+      <c r="A6" s="90" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="85" t="s">
-        <v>230</v>
+      <c r="A7" s="90" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="84" t="s">
-        <v>231</v>
+      <c r="A9" s="89" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="85" t="s">
-        <v>232</v>
+      <c r="A10" s="90" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="85" t="s">
-        <v>233</v>
+      <c r="A11" s="90" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="85" t="s">
-        <v>234</v>
+      <c r="A12" s="90" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="85" t="s">
-        <v>235</v>
+      <c r="A13" s="90" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="84" t="s">
-        <v>236</v>
+      <c r="A15" s="89" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="85" t="s">
-        <v>237</v>
+      <c r="A16" s="90" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="85" t="s">
-        <v>238</v>
+      <c r="A17" s="90" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="85" t="s">
-        <v>239</v>
+      <c r="A18" s="90" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="84" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="85" t="s">
-        <v>241</v>
+      <c r="A20" s="89" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="90" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="90" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="90" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="89" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="90" t="s">
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>